<commit_message>
#167 Updated Deliverables after Notes Section deletion.
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Bottom_Board_v3.4/BOM/Client BOM-LSS_Bottom_Board_v3.4.xlsx
+++ b/Design-Files/LSS_Bottom_Board_v3.4/BOM/Client BOM-LSS_Bottom_Board_v3.4.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\XPENDER\Documents\GitHub\ColeBenson-SmartMotors\Design-Files\LSS_Bottom_Board_v3.4\Project Outputs for LSS_Bottom_Board_v3.4\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiberDB\Documents\GitHub\ColeBenson-SmartMotors\Design-Files\LSS_Bottom_Board_v3.4\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="182">
   <si>
     <t>Description</t>
   </si>
@@ -561,14 +561,34 @@
   </si>
   <si>
     <t>RTD Temp Sensor</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>* Symbol is used for 0.1uF</t>
+  </si>
+  <si>
+    <t># Symbol is used for 10K</t>
+  </si>
+  <si>
+    <t>@ Symbol is used for 0R</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -590,7 +610,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -613,22 +633,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -669,7 +678,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -961,7 +991,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:H38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20.42578125" style="6" customWidth="1"/>
@@ -971,9 +1001,10 @@
     <col min="5" max="5" width="16.5703125" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" style="8" customWidth="1"/>
     <col min="7" max="7" width="16.5703125" style="11" customWidth="1"/>
+    <col min="8" max="8" width="34.140625" style="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>1</v>
       </c>
@@ -995,8 +1026,11 @@
       <c r="G1" s="9" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H1" s="19" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
@@ -1018,8 +1052,9 @@
       <c r="G2" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+      <c r="H2" s="20"/>
+    </row>
+    <row r="3" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>15</v>
       </c>
@@ -1041,8 +1076,11 @@
       <c r="G3" s="10">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H3" s="21" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>20</v>
       </c>
@@ -1064,8 +1102,9 @@
       <c r="G4" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H4" s="20"/>
+    </row>
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>26</v>
       </c>
@@ -1087,8 +1126,9 @@
       <c r="G5" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H5" s="20"/>
+    </row>
+    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>32</v>
       </c>
@@ -1110,8 +1150,9 @@
       <c r="G6" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H6" s="20"/>
+    </row>
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>37</v>
       </c>
@@ -1133,8 +1174,9 @@
       <c r="G7" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H7" s="20"/>
+    </row>
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>43</v>
       </c>
@@ -1156,8 +1198,9 @@
       <c r="G8" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+      <c r="H8" s="20"/>
+    </row>
+    <row r="9" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>48</v>
       </c>
@@ -1179,8 +1222,9 @@
       <c r="G9" s="10">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" ht="165" x14ac:dyDescent="0.25">
+      <c r="H9" s="20"/>
+    </row>
+    <row r="10" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>51</v>
       </c>
@@ -1202,8 +1246,9 @@
       <c r="G10" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H10" s="20"/>
+    </row>
+    <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>56</v>
       </c>
@@ -1225,8 +1270,9 @@
       <c r="G11" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="H11" s="20"/>
+    </row>
+    <row r="12" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>60</v>
       </c>
@@ -1248,8 +1294,9 @@
       <c r="G12" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H12" s="20"/>
+    </row>
+    <row r="13" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>64</v>
       </c>
@@ -1271,8 +1318,9 @@
       <c r="G13" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H13" s="20"/>
+    </row>
+    <row r="14" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>68</v>
       </c>
@@ -1294,8 +1342,9 @@
       <c r="G14" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" ht="150" x14ac:dyDescent="0.25">
+      <c r="H14" s="20"/>
+    </row>
+    <row r="15" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>73</v>
       </c>
@@ -1317,8 +1366,11 @@
       <c r="G15" s="10">
         <v>38</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H15" s="23" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>78</v>
       </c>
@@ -1340,8 +1392,11 @@
       <c r="G16" s="10">
         <v>7</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+      <c r="H16" s="21" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>83</v>
       </c>
@@ -1363,8 +1418,9 @@
       <c r="G17" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H17" s="20"/>
+    </row>
+    <row r="18" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>88</v>
       </c>
@@ -1386,8 +1442,9 @@
       <c r="G18" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H18" s="20"/>
+    </row>
+    <row r="19" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>92</v>
       </c>
@@ -1409,8 +1466,9 @@
       <c r="G19" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H19" s="20"/>
+    </row>
+    <row r="20" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>96</v>
       </c>
@@ -1432,8 +1490,9 @@
       <c r="G20" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H20" s="20"/>
+    </row>
+    <row r="21" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>101</v>
       </c>
@@ -1455,8 +1514,9 @@
       <c r="G21" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H21" s="20"/>
+    </row>
+    <row r="22" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>105</v>
       </c>
@@ -1478,8 +1538,9 @@
       <c r="G22" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H22" s="20"/>
+    </row>
+    <row r="23" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>109</v>
       </c>
@@ -1501,8 +1562,9 @@
       <c r="G23" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H23" s="20"/>
+    </row>
+    <row r="24" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>113</v>
       </c>
@@ -1524,8 +1586,9 @@
       <c r="G24" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H24" s="20"/>
+    </row>
+    <row r="25" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>117</v>
       </c>
@@ -1547,8 +1610,9 @@
       <c r="G25" s="10">
         <v>2</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+      <c r="H25" s="20"/>
+    </row>
+    <row r="26" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>121</v>
       </c>
@@ -1570,8 +1634,9 @@
       <c r="G26" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" ht="165" x14ac:dyDescent="0.25">
+      <c r="H26" s="20"/>
+    </row>
+    <row r="27" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>125</v>
       </c>
@@ -1591,8 +1656,9 @@
       <c r="G27" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H27" s="20"/>
+    </row>
+    <row r="28" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>129</v>
       </c>
@@ -1614,8 +1680,9 @@
       <c r="G28" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H28" s="20"/>
+    </row>
+    <row r="29" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>134</v>
       </c>
@@ -1637,8 +1704,9 @@
       <c r="G29" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H29" s="20"/>
+    </row>
+    <row r="30" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>139</v>
       </c>
@@ -1660,8 +1728,9 @@
       <c r="G30" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H30" s="20"/>
+    </row>
+    <row r="31" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>144</v>
       </c>
@@ -1683,8 +1752,9 @@
       <c r="G31" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H31" s="20"/>
+    </row>
+    <row r="32" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>148</v>
       </c>
@@ -1706,8 +1776,9 @@
       <c r="G32" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H32" s="20"/>
+    </row>
+    <row r="33" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>152</v>
       </c>
@@ -1729,8 +1800,9 @@
       <c r="G33" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H33" s="20"/>
+    </row>
+    <row r="34" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>157</v>
       </c>
@@ -1752,8 +1824,9 @@
       <c r="G34" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H34" s="20"/>
+    </row>
+    <row r="35" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>161</v>
       </c>
@@ -1775,8 +1848,9 @@
       <c r="G35" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H35" s="20"/>
+    </row>
+    <row r="36" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>166</v>
       </c>
@@ -1798,8 +1872,9 @@
       <c r="G36" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="H36" s="20"/>
+    </row>
+    <row r="37" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>171</v>
       </c>
@@ -1821,29 +1896,31 @@
       <c r="G37" s="10">
         <v>1</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="6" t="s">
+      <c r="H37" s="20"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
         <v>176</v>
       </c>
-      <c r="B38" s="15" t="s">
+      <c r="B38" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="C38" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="D38" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="E38" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="F38" s="16" t="s">
-        <v>174</v>
-      </c>
-      <c r="G38" s="16" t="s">
-        <v>174</v>
-      </c>
+      <c r="C38" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="D38" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="E38" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="F38" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="G38" s="18" t="s">
+        <v>174</v>
+      </c>
+      <c r="H38" s="20"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D1:D37 D39:D1048576">

</xml_diff>

<commit_message>
#167  Updated Deliverables of Top Board deletion of Notes from PCB.
</commit_message>
<xml_diff>
--- a/Design-Files/LSS_Bottom_Board_v3.4/BOM/Client BOM-LSS_Bottom_Board_v3.4.xlsx
+++ b/Design-Files/LSS_Bottom_Board_v3.4/BOM/Client BOM-LSS_Bottom_Board_v3.4.xlsx
@@ -566,13 +566,13 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>* Symbol is used for 0.1uF</t>
-  </si>
-  <si>
-    <t># Symbol is used for 10K</t>
-  </si>
-  <si>
-    <t>@ Symbol is used for 0R</t>
+    <t>* Symbol is used for 0.1uF in PCB</t>
+  </si>
+  <si>
+    <t>@ Symbol is used for 0R in PCB</t>
+  </si>
+  <si>
+    <t># Symbol is used for 10K in PCB</t>
   </si>
 </sst>
 </file>
@@ -1001,7 +1001,7 @@
     <col min="5" max="5" width="16.5703125" customWidth="1"/>
     <col min="6" max="6" width="16.5703125" style="8" customWidth="1"/>
     <col min="7" max="7" width="16.5703125" style="11" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" style="22" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="43.28515625" style="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
@@ -1367,7 +1367,7 @@
         <v>38</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="45" x14ac:dyDescent="0.25">
@@ -1393,7 +1393,7 @@
         <v>7</v>
       </c>
       <c r="H16" s="21" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="90" x14ac:dyDescent="0.25">

</xml_diff>